<commit_message>
Update awards display order
</commit_message>
<xml_diff>
--- a/data/learning_portfolio.xlsx
+++ b/data/learning_portfolio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\88_YuHui\Streamlit\Richard_streamlit\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{711151BE-6D95-4C00-A498-6F73CADD12BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69C2246-5C86-4B2B-AEBB-8481441B6AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3793,16 +3793,16 @@
         <v>153</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="E7" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="F7" t="s">
         <v>169</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="J7" t="s">
         <v>36</v>
@@ -3897,16 +3897,16 @@
         <v>153</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="E11" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="F11" t="s">
         <v>169</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="J11" t="s">
         <v>36</v>
@@ -3915,10 +3915,10 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="C2 C3:C200" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="C2:C7 C8:C200" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"English,Math,Art,Science,Sports,Music,School,Community,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J2 J3:J200" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" sqref="J2:J7 J8:J200" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update Horizon Field Day event names
</commit_message>
<xml_diff>
--- a/data/learning_portfolio.xlsx
+++ b/data/learning_portfolio.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\88_YuHui\Streamlit\Richard_streamlit\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YuHui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69C2246-5C86-4B2B-AEBB-8481441B6AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3B25C0-289E-4F73-BF2B-C4AF62593B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="169">
   <si>
     <t>Field</t>
   </si>
@@ -514,19 +514,19 @@
     <t>Richard was selected to lead the athletes' oath at Horizon Field Day, representing fellow participants and highlighting sportsmanship and fair play.</t>
   </si>
   <si>
-    <t>Horizon Field Day – Rope Skipping (G4 Boys)</t>
+    <t>Horizon Field Day – Jump Rope (G4 Boys)</t>
   </si>
   <si>
     <t>1st Place</t>
   </si>
   <si>
-    <t>Richard won first place in the Grade 4 boys' rope skipping event at Horizon Field Day, demonstrating coordination, speed, and focus.</t>
-  </si>
-  <si>
-    <t>Horizon Field Day – Long Jump (G4 Boys)</t>
-  </si>
-  <si>
-    <t>Richard won first place in the Grade 4 boys' long jump event at Horizon Field Day, showing determination and athletic ability.</t>
+    <t>Richard won first place in the Grade 4 boys' jump rope event at Horizon Field Day, demonstrating coordination, speed, and focus.</t>
+  </si>
+  <si>
+    <t>Horizon Field Day – Standing Long Jump (G4 Boys)</t>
+  </si>
+  <si>
+    <t>Richard won first place in the Grade 4 boys' standing long jump event at Horizon Field Day, showing determination and athletic ability.</t>
   </si>
   <si>
     <t>Horizon Field Day – Shuttle Run (G4 Boys)</t>
@@ -535,24 +535,19 @@
     <t>Richard won first place in the Grade 4 boys' shuttle run event at Horizon Field Day, demonstrating speed, agility, and focus.</t>
   </si>
   <si>
-    <t>Horizon Field Day – Softball Throw (G4 Boys)</t>
-  </si>
-  <si>
-    <t>Richard won first place in the Grade 4 boys' softball throw event at Horizon Field Day, demonstrating strength, technique, and concentration.</t>
+    <t>Horizon Field Day – Ball Throw (G4 Boys)</t>
+  </si>
+  <si>
+    <t>Richard won first place in the Grade 4 boys' ball throw event at Horizon Field Day, demonstrating strength, technique, and concentration.</t>
+  </si>
+  <si>
+    <t>Horizon Field Day – Boys' MVP</t>
   </si>
   <si>
     <t>Boys' MVP</t>
   </si>
   <si>
     <t>Richard was named Boys' MVP at Horizon Field Day in recognition of his outstanding overall performance across the sporting events.</t>
-  </si>
-  <si>
-    <t>Horizon Field Day – Boys' MVP</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>Horizon</t>
-    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -3793,16 +3788,13 @@
         <v>153</v>
       </c>
       <c r="D7" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="E7" t="s">
+        <v>167</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>168</v>
-      </c>
-      <c r="E7" t="s">
-        <v>166</v>
-      </c>
-      <c r="F7" t="s">
-        <v>169</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>167</v>
       </c>
       <c r="J7" t="s">
         <v>36</v>
@@ -3824,9 +3816,6 @@
       <c r="E8" t="s">
         <v>158</v>
       </c>
-      <c r="F8" t="s">
-        <v>169</v>
-      </c>
       <c r="G8" s="13" t="s">
         <v>161</v>
       </c>
@@ -3845,16 +3834,13 @@
         <v>153</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E9" t="s">
         <v>158</v>
       </c>
-      <c r="F9" t="s">
-        <v>169</v>
-      </c>
       <c r="G9" s="13" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="J9" t="s">
         <v>36</v>
@@ -3871,16 +3857,13 @@
         <v>153</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E10" t="s">
         <v>158</v>
       </c>
-      <c r="F10" t="s">
-        <v>169</v>
-      </c>
       <c r="G10" s="13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="J10" t="s">
         <v>36</v>
@@ -3902,9 +3885,6 @@
       <c r="E11" t="s">
         <v>158</v>
       </c>
-      <c r="F11" t="s">
-        <v>169</v>
-      </c>
       <c r="G11" s="13" t="s">
         <v>159</v>
       </c>
@@ -3915,10 +3895,10 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="C2:C7 C8:C200" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="C11:C200 C2:C10" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"English,Math,Art,Science,Sports,Music,School,Community,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J2:J7 J8:J200" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" sqref="J11:J200 J2:J10" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add DELF certificate and The Last Bear reading record
</commit_message>
<xml_diff>
--- a/data/learning_portfolio.xlsx
+++ b/data/learning_portfolio.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YuHui\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\88_YuHui\Streamlit\Richard_streamlit\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3B25C0-289E-4F73-BF2B-C4AF62593B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ACAB9BC-5029-4498-9743-4DE8663377BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Profile" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="175">
   <si>
     <t>Field</t>
   </si>
@@ -205,36 +205,9 @@
     <t>project_001.jpg</t>
   </si>
   <si>
-    <t>Art</t>
-  </si>
-  <si>
-    <t>My Favorite Animal Drawing</t>
-  </si>
-  <si>
-    <t>An illustrated animal drawing with a short description.</t>
-  </si>
-  <si>
-    <t>Color pencils</t>
-  </si>
-  <si>
-    <t>project_002.jpg</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Science</t>
   </si>
   <si>
-    <t>Mini Weather Chart</t>
-  </si>
-  <si>
-    <t>Recorded weather changes and summarized temperature patterns.</t>
-  </si>
-  <si>
-    <t>Notebook, chart</t>
-  </si>
-  <si>
     <t>BookTitle</t>
   </si>
   <si>
@@ -244,310 +217,371 @@
     <t>Rating</t>
   </si>
   <si>
-    <t>Amazing Insects</t>
-  </si>
-  <si>
-    <t>Sample Author</t>
-  </si>
-  <si>
-    <t>I learned that insects use many ways to protect themselves.</t>
+    <t>Story</t>
+  </si>
+  <si>
+    <t>book_002.jpg</t>
+  </si>
+  <si>
+    <t>English</t>
+  </si>
+  <si>
+    <t>Reading</t>
+  </si>
+  <si>
+    <t>Expression</t>
+  </si>
+  <si>
+    <t>SelfLearning</t>
+  </si>
+  <si>
+    <t>Creativity</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Started building regular reading habits.</t>
+  </si>
+  <si>
+    <t>More confident in sharing ideas and completing projects.</t>
+  </si>
+  <si>
+    <t>Shows stronger curiosity, expression, and independent learning.</t>
+  </si>
+  <si>
+    <t>MostImportantProgress</t>
+  </si>
+  <si>
+    <t>FavoriteProject</t>
+  </si>
+  <si>
+    <t>ImportantAwards</t>
+  </si>
+  <si>
+    <t>NextYearGoals</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>CoverImage</t>
+  </si>
+  <si>
+    <t>More confident speaking and presenting in front of others.</t>
+  </si>
+  <si>
+    <t>English Reading Contest - Second Place</t>
+  </si>
+  <si>
+    <t>Read more English books and complete two science projects.</t>
+  </si>
+  <si>
+    <t>A year of steady growth in reading, expression, and creativity.</t>
+  </si>
+  <si>
+    <t>review_2026.jpg</t>
+  </si>
+  <si>
+    <t>Built a stronger reading routine.</t>
+  </si>
+  <si>
+    <t>Animal Drawing Project</t>
+  </si>
+  <si>
+    <t>Creative Drawing Challenge - Excellent Work</t>
+  </si>
+  <si>
+    <t>Practice English speaking and keep a weekly reading log.</t>
+  </si>
+  <si>
+    <t>A year of building habits and discovering interests.</t>
+  </si>
+  <si>
+    <t>AllowedValues</t>
+  </si>
+  <si>
+    <t>Usage</t>
+  </si>
+  <si>
+    <t>Learning Category</t>
+  </si>
+  <si>
+    <t>Used in LearningTimeline.Category</t>
+  </si>
+  <si>
+    <t>Award Category</t>
+  </si>
+  <si>
+    <t>Used in Awards.Category</t>
+  </si>
+  <si>
+    <t>Project Category</t>
+  </si>
+  <si>
+    <t>Coding, Art, Science, Writing, Music, Video, Presentation, Other</t>
+  </si>
+  <si>
+    <t>Used in Projects.Category</t>
+  </si>
+  <si>
+    <t>Yes, No</t>
+  </si>
+  <si>
+    <t>Show item on the home page</t>
+  </si>
+  <si>
+    <t>Public-safe, Private</t>
+  </si>
+  <si>
+    <t>Use Public-safe for items that can be shared</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 4, 5</t>
+  </si>
+  <si>
+    <t>ReadingLog.Rating</t>
+  </si>
+  <si>
+    <t>Richard's Learning Journey - Data Dashboard</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Total Learning Records</t>
+  </si>
+  <si>
+    <t>Featured Learning Records</t>
+  </si>
+  <si>
+    <t>Total Awards</t>
+  </si>
+  <si>
+    <t>Total Projects</t>
+  </si>
+  <si>
+    <t>Total Books</t>
+  </si>
+  <si>
+    <t>Average Reading Rating</t>
+  </si>
+  <si>
+    <t>Public-safe</t>
+  </si>
+  <si>
+    <t>Camp</t>
+  </si>
+  <si>
+    <t>Mario Detective &amp; Coin-Earning Little Boss Camp</t>
+  </si>
+  <si>
+    <t>Richard joined a playful camp that combined detective-style problem solving with money-themed activities. The experience helped him practice observation, logical thinking, decision-making, and basic financial awareness.</t>
+  </si>
+  <si>
+    <t>I practiced solving clues, making choices, and learning how to think like a little boss.</t>
+  </si>
+  <si>
+    <t>Musical Theatre Camp</t>
+  </si>
+  <si>
+    <t>Richard participated in a musical theatre camp and explored singing, movement, acting, and stage expression. The experience helped him build confidence, creativity, teamwork, and presentation skills.</t>
+  </si>
+  <si>
+    <t>I enjoyed expressing myself through music, movement, and performance.</t>
+  </si>
+  <si>
+    <t>Plant growth observation</t>
+  </si>
+  <si>
+    <t>Observed how light and water affect plant growth.</t>
+  </si>
+  <si>
+    <t>I learned to record small changes every day.</t>
+  </si>
+  <si>
+    <t>French</t>
+  </si>
+  <si>
+    <t>DELF Prim A1.1 Certificate Presentation</t>
+  </si>
+  <si>
+    <t>After passing the DELF Prim A1.1 French language examination in April 2026, Richard received his certificate from the president of Alliance Française de Taiwan on September 17, 2026.</t>
+  </si>
+  <si>
+    <t>SMC Regional Round</t>
+  </si>
+  <si>
+    <t>Marshall Cavendish Education (MCE)</t>
+  </si>
+  <si>
+    <t>Richard earned a Silver Award in the SMC Regional Round. The competition encouraged him to think carefully, stay focused, and challenge himself in mathematics.</t>
+  </si>
+  <si>
+    <t>award_002.jpg</t>
+  </si>
+  <si>
+    <t>Sports</t>
+  </si>
+  <si>
+    <t>Horizon Field Day – Boys' MVP</t>
+  </si>
+  <si>
+    <t>Boys' MVP</t>
+  </si>
+  <si>
+    <t>Richard was named Boys' MVP at Horizon Field Day in recognition of his outstanding overall performance across the sporting events.</t>
+  </si>
+  <si>
+    <t>Horizon Field Day – Athlete's Oath</t>
+  </si>
+  <si>
+    <t>Athlete's Oath Representative</t>
+  </si>
+  <si>
+    <t>Richard was selected to lead the athletes' oath at Horizon Field Day, representing fellow participants and highlighting sportsmanship and fair play.</t>
+  </si>
+  <si>
+    <t>Horizon Field Day – Standing Long Jump (G4 Boys)</t>
+  </si>
+  <si>
+    <t>1st Place</t>
+  </si>
+  <si>
+    <t>Richard won first place in the Grade 4 boys' standing long jump event at Horizon Field Day, showing determination and athletic ability.</t>
+  </si>
+  <si>
+    <t>Horizon Field Day – Shuttle Run (G4 Boys)</t>
+  </si>
+  <si>
+    <t>Richard won first place in the Grade 4 boys' shuttle run event at Horizon Field Day, demonstrating speed, agility, and focus.</t>
+  </si>
+  <si>
+    <t>Horizon Field Day – Ball Throw (G4 Boys)</t>
+  </si>
+  <si>
+    <t>Richard won first place in the Grade 4 boys' ball throw event at Horizon Field Day, demonstrating strength, technique, and concentration.</t>
+  </si>
+  <si>
+    <t>Horizon Field Day – Jump Rope (G4 Boys)</t>
+  </si>
+  <si>
+    <t>Richard won first place in the Grade 4 boys' jump rope event at Horizon Field Day, demonstrating coordination, speed, and focus.</t>
+  </si>
+  <si>
+    <t>DELF Prim A1.1 French Language Examination</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Alliance Française de Taiwan</t>
+  </si>
+  <si>
+    <t>Richard passed the DELF Prim A1.1 French language examination in April 2026. On September 17, 2026, he received his certificate from the president of Alliance Française de Taiwan.</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>The Last Bear</t>
+  </si>
+  <si>
+    <t>Hannah Gold</t>
+  </si>
+  <si>
+    <t>Reading, School Activity, Science, English, French, Math, Art, Music, Sports, Coding, Life Skill, Other</t>
+  </si>
+  <si>
+    <t>English, French, Math, Art, Science, Sports, Music, School, Community, Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> City Building, Energy, and Creativity</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Richard designed and built a creative city model with roads, railways, buildings, wind turbines, and solar panels. Through this project, he explored how a city works and learned about renewable energy, transportation, planning, and teamwork.</t>
+  </si>
+  <si>
+    <t>The Explorer</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Katherine Rundell</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Story</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>book_004.jpg</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Wayside School</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Louis Sachar</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>book_001.jpg</t>
-  </si>
-  <si>
-    <t>The Little Explorer</t>
-  </si>
-  <si>
-    <t>Story</t>
-  </si>
-  <si>
-    <t>The story reminded me to keep trying even when something is difficult.</t>
-  </si>
-  <si>
-    <t>Space for Kids</t>
-  </si>
-  <si>
-    <t>My favorite topic was planets.</t>
-  </si>
-  <si>
-    <t>book_002.jpg</t>
-  </si>
-  <si>
-    <t>English</t>
-  </si>
-  <si>
-    <t>Reading</t>
-  </si>
-  <si>
-    <t>Expression</t>
-  </si>
-  <si>
-    <t>SelfLearning</t>
-  </si>
-  <si>
-    <t>Creativity</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Started building regular reading habits.</t>
-  </si>
-  <si>
-    <t>More confident in sharing ideas and completing projects.</t>
-  </si>
-  <si>
-    <t>Shows stronger curiosity, expression, and independent learning.</t>
-  </si>
-  <si>
-    <t>MostImportantProgress</t>
-  </si>
-  <si>
-    <t>FavoriteProject</t>
-  </si>
-  <si>
-    <t>ImportantAwards</t>
-  </si>
-  <si>
-    <t>NextYearGoals</t>
-  </si>
-  <si>
-    <t>Summary</t>
-  </si>
-  <si>
-    <t>CoverImage</t>
-  </si>
-  <si>
-    <t>More confident speaking and presenting in front of others.</t>
-  </si>
-  <si>
-    <t>English Reading Contest - Second Place</t>
-  </si>
-  <si>
-    <t>Read more English books and complete two science projects.</t>
-  </si>
-  <si>
-    <t>A year of steady growth in reading, expression, and creativity.</t>
-  </si>
-  <si>
-    <t>review_2026.jpg</t>
-  </si>
-  <si>
-    <t>Built a stronger reading routine.</t>
-  </si>
-  <si>
-    <t>Animal Drawing Project</t>
-  </si>
-  <si>
-    <t>Creative Drawing Challenge - Excellent Work</t>
-  </si>
-  <si>
-    <t>Practice English speaking and keep a weekly reading log.</t>
-  </si>
-  <si>
-    <t>A year of building habits and discovering interests.</t>
-  </si>
-  <si>
-    <t>AllowedValues</t>
-  </si>
-  <si>
-    <t>Usage</t>
-  </si>
-  <si>
-    <t>Learning Category</t>
-  </si>
-  <si>
-    <t>Reading, School Activity, Science, English, Math, Art, Music, Sports, Coding, Life Skill, Other</t>
-  </si>
-  <si>
-    <t>Used in LearningTimeline.Category</t>
-  </si>
-  <si>
-    <t>Award Category</t>
-  </si>
-  <si>
-    <t>English, Math, Art, Science, Sports, Music, School, Community, Other</t>
-  </si>
-  <si>
-    <t>Used in Awards.Category</t>
-  </si>
-  <si>
-    <t>Project Category</t>
-  </si>
-  <si>
-    <t>Coding, Art, Science, Writing, Music, Video, Presentation, Other</t>
-  </si>
-  <si>
-    <t>Used in Projects.Category</t>
-  </si>
-  <si>
-    <t>Yes, No</t>
-  </si>
-  <si>
-    <t>Show item on the home page</t>
-  </si>
-  <si>
-    <t>Public-safe, Private</t>
-  </si>
-  <si>
-    <t>Use Public-safe for items that can be shared</t>
-  </si>
-  <si>
-    <t>1, 2, 3, 4, 5</t>
-  </si>
-  <si>
-    <t>ReadingLog.Rating</t>
-  </si>
-  <si>
-    <t>Richard's Learning Journey - Data Dashboard</t>
-  </si>
-  <si>
-    <t>Metric</t>
-  </si>
-  <si>
-    <t>Formula</t>
-  </si>
-  <si>
-    <t>Total Learning Records</t>
-  </si>
-  <si>
-    <t>Featured Learning Records</t>
-  </si>
-  <si>
-    <t>Total Awards</t>
-  </si>
-  <si>
-    <t>Total Projects</t>
-  </si>
-  <si>
-    <t>Total Books</t>
-  </si>
-  <si>
-    <t>Average Reading Rating</t>
-  </si>
-  <si>
-    <t>Finished an animal science book</t>
-  </si>
-  <si>
-    <t>Learned how insects adapt to different environments.</t>
-  </si>
-  <si>
-    <t>My favorite part was learning about beetles.</t>
-  </si>
-  <si>
-    <t>learning_001.jpg</t>
-  </si>
-  <si>
-    <t>Public-safe</t>
-  </si>
-  <si>
-    <t>School Activity</t>
-  </si>
-  <si>
-    <t>Class presentation practice</t>
-  </si>
-  <si>
-    <t>Practiced speaking clearly and organizing ideas.</t>
-  </si>
-  <si>
-    <t>I felt more confident after practicing.</t>
-  </si>
-  <si>
-    <t>Private</t>
-  </si>
-  <si>
-    <t>Camp</t>
-  </si>
-  <si>
-    <t>Mario Detective &amp; Coin-Earning Little Boss Camp</t>
-  </si>
-  <si>
-    <t>Richard joined a playful camp that combined detective-style problem solving with money-themed activities. The experience helped him practice observation, logical thinking, decision-making, and basic financial awareness.</t>
-  </si>
-  <si>
-    <t>I practiced solving clues, making choices, and learning how to think like a little boss.</t>
-  </si>
-  <si>
-    <t>Musical Theatre Camp</t>
-  </si>
-  <si>
-    <t>Richard participated in a musical theatre camp and explored singing, movement, acting, and stage expression. The experience helped him build confidence, creativity, teamwork, and presentation skills.</t>
-  </si>
-  <si>
-    <t>I enjoyed expressing myself through music, movement, and performance.</t>
-  </si>
-  <si>
-    <t>Plant growth observation</t>
-  </si>
-  <si>
-    <t>Observed how light and water affect plant growth.</t>
-  </si>
-  <si>
-    <t>I learned to record small changes every day.</t>
-  </si>
-  <si>
-    <t>learning_002.jpg</t>
-  </si>
-  <si>
-    <t>SMC Regional Round</t>
-  </si>
-  <si>
-    <t>Marshall Cavendish Education (MCE)</t>
-  </si>
-  <si>
-    <t>Richard earned a Silver Award in the SMC Regional Round. The competition encouraged him to think carefully, stay focused, and challenge himself in mathematics.</t>
-  </si>
-  <si>
-    <t>award_002.jpg</t>
-  </si>
-  <si>
-    <t>Sports</t>
-  </si>
-  <si>
-    <t>Horizon Field Day – Athlete's Oath</t>
-  </si>
-  <si>
-    <t>Athlete's Oath Representative</t>
-  </si>
-  <si>
-    <t>Richard was selected to lead the athletes' oath at Horizon Field Day, representing fellow participants and highlighting sportsmanship and fair play.</t>
-  </si>
-  <si>
-    <t>Horizon Field Day – Jump Rope (G4 Boys)</t>
-  </si>
-  <si>
-    <t>1st Place</t>
-  </si>
-  <si>
-    <t>Richard won first place in the Grade 4 boys' jump rope event at Horizon Field Day, demonstrating coordination, speed, and focus.</t>
-  </si>
-  <si>
-    <t>Horizon Field Day – Standing Long Jump (G4 Boys)</t>
-  </si>
-  <si>
-    <t>Richard won first place in the Grade 4 boys' standing long jump event at Horizon Field Day, showing determination and athletic ability.</t>
-  </si>
-  <si>
-    <t>Horizon Field Day – Shuttle Run (G4 Boys)</t>
-  </si>
-  <si>
-    <t>Richard won first place in the Grade 4 boys' shuttle run event at Horizon Field Day, demonstrating speed, agility, and focus.</t>
-  </si>
-  <si>
-    <t>Horizon Field Day – Ball Throw (G4 Boys)</t>
-  </si>
-  <si>
-    <t>Richard won first place in the Grade 4 boys' ball throw event at Horizon Field Day, demonstrating strength, technique, and concentration.</t>
-  </si>
-  <si>
-    <t>Horizon Field Day – Boys' MVP</t>
-  </si>
-  <si>
-    <t>Boys' MVP</t>
-  </si>
-  <si>
-    <t>Richard was named Boys' MVP at Horizon Field Day in recognition of his outstanding overall performance across the sporting events.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>The Wild Robot</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Peter Brown</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>The Wild Robot Escapes</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>book_003.jpg</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>The Last Bear.jpg</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Film Camp</t>
+  </si>
+  <si>
+    <t>Richard joined a film camp and explored storytelling, acting, camera work, and creative expression. The experience helped him develop imagination, communication skills, teamwork, and confidence in presenting ideas.</t>
+  </si>
+  <si>
+    <t>I enjoyed creating stories, acting with others, and learning how ideas can become a film.</t>
+  </si>
+  <si>
+    <t>A Star Multi Sport Camp</t>
+  </si>
+  <si>
+    <t>Richard participated in a multi-sport camp and experienced different physical activities through games, teamwork, and practice. The camp helped him develop coordination, confidence, sportsmanship, and perseverance.</t>
+  </si>
+  <si>
+    <t>I tried different sports, practiced with others, and learned to keep going even when the activities were challenging.</t>
+  </si>
+  <si>
+    <t>Flight Camp</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Richard participated in a flight camp that introduced the roles of pilots and cabin crew through hands-on training activities. The experience helped him understand aviation teamwork, safety, communication, and responsibility</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>I enjoyed learning about pilots and cabin crew, and I discovered how teamwork and responsibility are important in aviation.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -557,7 +591,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -584,6 +618,11 @@
       <family val="3"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -608,7 +647,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -616,12 +655,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -660,10 +710,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -693,7 +750,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="LearningTimelineTable" displayName="LearningTimelineTable" ref="A1:J4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="LearningTimelineTable" displayName="LearningTimelineTable" ref="A1:J5">
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Date"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Year"/>
@@ -747,7 +804,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="ReadingLogTable" displayName="ReadingLogTable" ref="A1:I4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="ReadingLogTable" displayName="ReadingLogTable" ref="A1:I6">
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Date"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Year"/>
@@ -1052,7 +1109,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J200"/>
+  <dimension ref="A1:J201"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1097,110 +1154,108 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="6">
-        <v>46174</v>
-      </c>
-      <c r="B2" s="8">
-        <v>2026</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>128</v>
+    <row r="2" spans="1:10" ht="57">
+      <c r="A2" s="18">
+        <v>45887</v>
+      </c>
+      <c r="B2" s="13">
+        <v>2025</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>166</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>129</v>
+        <v>167</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="J2" s="10" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="6">
-        <v>46162</v>
-      </c>
-      <c r="B3" s="8">
-        <v>2026</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>134</v>
+      <c r="J2" s="13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="57">
+      <c r="A3" s="18">
+        <v>45999</v>
+      </c>
+      <c r="B3" s="13">
+        <v>2025</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>169</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>135</v>
+        <v>170</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>137</v>
+        <v>171</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="57">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
+        <v>46006</v>
+      </c>
+      <c r="B4" s="4">
+        <v>2025</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="57">
+      <c r="A5" s="6">
         <v>46146</v>
-      </c>
-      <c r="B4" s="8">
-        <v>2026</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="42.75">
-      <c r="A5" s="6">
-        <v>46125</v>
       </c>
       <c r="B5" s="8">
         <v>2026</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>142</v>
+        <v>111</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>143</v>
+        <v>112</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>144</v>
+        <v>113</v>
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="10"/>
@@ -1208,62 +1263,90 @@
         <v>36</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="42.75">
       <c r="A6" s="6">
-        <v>46124</v>
+        <v>46125</v>
       </c>
       <c r="B6" s="8">
         <v>2026</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>145</v>
+        <v>114</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>146</v>
+        <v>115</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>148</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="G6" s="10"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10" t="s">
         <v>36</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="11"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="11"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
+      <c r="A7" s="6">
+        <v>46124</v>
+      </c>
+      <c r="B7" s="8">
+        <v>2026</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="42.75">
+      <c r="A8" s="11">
+        <v>46282</v>
+      </c>
+      <c r="B8" s="12">
+        <v>2026</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>122</v>
+      </c>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="13"/>
+      <c r="I8" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11"/>
@@ -3569,16 +3652,28 @@
       <c r="I200" s="13"/>
       <c r="J200" s="13"/>
     </row>
+    <row r="201" spans="1:10">
+      <c r="A201" s="11"/>
+      <c r="B201" s="12"/>
+      <c r="C201" s="13"/>
+      <c r="D201" s="13"/>
+      <c r="E201" s="13"/>
+      <c r="F201" s="13"/>
+      <c r="G201" s="13"/>
+      <c r="H201" s="13"/>
+      <c r="I201" s="13"/>
+      <c r="J201" s="13"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations count="3">
-    <dataValidation type="list" sqref="C2:C200" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <dataValidations disablePrompts="1" count="3">
+    <dataValidation type="list" sqref="C2:C201" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Reading,School Activity,Science,English,Math,Art,Music,Sports,Coding,Life Skill,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="I2:I200" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" sqref="I2:I201" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J2:J200" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" sqref="J2:J201" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Public-safe,Private"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3591,7 +3686,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -3735,19 +3830,19 @@
         <v>31</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>38</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>150</v>
+        <v>124</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>151</v>
+        <v>125</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>152</v>
+        <v>126</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4" t="s">
@@ -3762,16 +3857,16 @@
         <v>2026</v>
       </c>
       <c r="C6" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="E6" t="s">
-        <v>155</v>
+        <v>129</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>156</v>
+        <v>130</v>
       </c>
       <c r="J6" t="s">
         <v>36</v>
@@ -3785,16 +3880,16 @@
         <v>2026</v>
       </c>
       <c r="C7" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>166</v>
+        <v>131</v>
       </c>
       <c r="E7" t="s">
-        <v>167</v>
+        <v>132</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>168</v>
+        <v>133</v>
       </c>
       <c r="J7" t="s">
         <v>36</v>
@@ -3808,16 +3903,16 @@
         <v>2026</v>
       </c>
       <c r="C8" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>160</v>
+        <v>134</v>
       </c>
       <c r="E8" t="s">
-        <v>158</v>
+        <v>135</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>161</v>
+        <v>136</v>
       </c>
       <c r="J8" t="s">
         <v>36</v>
@@ -3831,16 +3926,16 @@
         <v>2026</v>
       </c>
       <c r="C9" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>164</v>
+        <v>137</v>
       </c>
       <c r="E9" t="s">
-        <v>158</v>
+        <v>135</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>165</v>
+        <v>138</v>
       </c>
       <c r="J9" t="s">
         <v>36</v>
@@ -3854,16 +3949,16 @@
         <v>2026</v>
       </c>
       <c r="C10" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>162</v>
+        <v>139</v>
       </c>
       <c r="E10" t="s">
-        <v>158</v>
+        <v>135</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
       <c r="J10" t="s">
         <v>36</v>
@@ -3877,28 +3972,54 @@
         <v>2026</v>
       </c>
       <c r="C11" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="E11" t="s">
-        <v>158</v>
+        <v>135</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>159</v>
+        <v>142</v>
       </c>
       <c r="J11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="7">
+        <v>46282</v>
+      </c>
+      <c r="B12">
+        <v>2026</v>
+      </c>
+      <c r="C12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" t="s">
+        <v>143</v>
+      </c>
+      <c r="E12" t="s">
+        <v>144</v>
+      </c>
+      <c r="F12" t="s">
+        <v>145</v>
+      </c>
+      <c r="G12" t="s">
+        <v>146</v>
+      </c>
+      <c r="J12" t="s">
         <v>36</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="C11:C200 C2:C10" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="C2 C3:C200" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"English,Math,Art,Science,Sports,Music,School,Community,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J11:J200 J2:J10" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" sqref="J2 J3:J200" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3956,25 +4077,23 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="28.5">
+    <row r="2" spans="1:10" ht="71.25">
       <c r="A2" s="5">
-        <v>46181</v>
+        <v>46121</v>
       </c>
       <c r="B2" s="4">
         <v>2026</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>50</v>
+        <v>152</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>52</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="F2" s="4"/>
       <c r="G2" s="4" t="s">
         <v>53</v>
       </c>
@@ -3984,59 +4103,43 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" ht="28.5">
       <c r="A3" s="5">
-        <v>46137</v>
+        <v>46181</v>
       </c>
       <c r="B3" s="4">
         <v>2026</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>58</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="28.5">
-      <c r="A4" s="5">
-        <v>46086</v>
-      </c>
-      <c r="B4" s="4">
-        <v>2026</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>63</v>
-      </c>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="5"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
-      <c r="J4" s="4" t="s">
-        <v>36</v>
-      </c>
+      <c r="J4" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -4057,7 +4160,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -4079,10 +4182,10 @@
         <v>20</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>21</v>
@@ -4091,7 +4194,7 @@
         <v>23</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>24</v>
@@ -4102,87 +4205,137 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="5">
-        <v>46174</v>
+        <v>45908</v>
       </c>
       <c r="B2" s="4">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>67</v>
+        <v>154</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>68</v>
+        <v>155</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>69</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="F2" s="4"/>
       <c r="G2" s="4">
         <v>5</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>70</v>
+        <v>157</v>
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="28.5">
+    <row r="3" spans="1:9">
       <c r="A3" s="5">
-        <v>46156</v>
+        <v>45658</v>
       </c>
       <c r="B3" s="4">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>71</v>
+        <v>158</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>68</v>
+        <v>159</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>73</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="F3" s="4"/>
       <c r="G3" s="4">
-        <v>4</v>
-      </c>
-      <c r="H3" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>160</v>
+      </c>
       <c r="I3" s="4"/>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="5">
-        <v>46115</v>
+        <v>46027</v>
       </c>
       <c r="B4" s="4">
         <v>2026</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>74</v>
+        <v>161</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>68</v>
+        <v>162</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>75</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="F4" s="4"/>
       <c r="G4" s="4">
         <v>5</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="I4" s="4"/>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="5">
+        <v>46153</v>
+      </c>
+      <c r="B5" s="4">
+        <v>2026</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4">
+        <v>5</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="I5" s="4"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2026</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4">
+        <v>5</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="I6" s="4"/>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="14"/>
+      <c r="E7" s="17"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="G2:G200" xr:uid="{00000000-0002-0000-0400-000000000000}">
+    <dataValidation type="list" sqref="G2:G202" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4211,25 +4364,25 @@
         <v>20</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -4255,7 +4408,7 @@
         <v>4</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -4281,7 +4434,7 @@
         <v>4</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -4307,7 +4460,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -4338,22 +4491,22 @@
         <v>20</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.5">
@@ -4361,22 +4514,22 @@
         <v>2026</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>50</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -4384,19 +4537,19 @@
         <v>2025</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="G3" s="4"/>
     </row>
@@ -4424,43 +4577,43 @@
         <v>21</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="28.5">
       <c r="A2" s="4" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>105</v>
+        <v>150</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="28.5">
       <c r="A3" s="4" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>108</v>
+        <v>151</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -4468,10 +4621,10 @@
         <v>26</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -4479,21 +4632,21 @@
         <v>27</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="4" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>118</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -4515,75 +4668,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="20.25">
-      <c r="A1" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
+      <c r="A1" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="3" spans="1:6" ht="15">
       <c r="A3" s="1" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(LearningTimeline!D2:D200)</f>
-        <v>5</v>
+        <f>COUNTA(LearningTimeline!D2:D201)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF(LearningTimeline!I2:I200,"Yes")</f>
-        <v>4</v>
+        <f>COUNTIF(LearningTimeline!I2:I201,"Yes")</f>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="B6" s="3">
         <f>COUNTA(Awards!D2:D200)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="B7" s="3">
         <f>COUNTA(Projects!D2:D200)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="B8" s="3">
-        <f>COUNTA(ReadingLog!C2:C200)</f>
-        <v>3</v>
+        <f>COUNTA(ReadingLog!C7:C202)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="B9" s="3">
-        <f>IFERROR(AVERAGE(ReadingLog!G2:G200),0)</f>
-        <v>4.666666666666667</v>
+        <f>IFERROR(AVERAGE(ReadingLog!G7:G202),0)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Richard learning portfolio
</commit_message>
<xml_diff>
--- a/data/learning_portfolio.xlsx
+++ b/data/learning_portfolio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\88_YuHui\Streamlit\Richard_streamlit\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ACAB9BC-5029-4498-9743-4DE8663377BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800E0365-15B6-45F7-AC74-A30D4329A28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Profile" sheetId="1" r:id="rId1"/>
@@ -550,10 +550,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>The Last Bear.jpg</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>Film Camp</t>
   </si>
   <si>
@@ -581,6 +577,10 @@
   </si>
   <si>
     <t>I enjoyed learning about pilots and cabin crew, and I discovered how teamwork and responsibility are important in aviation.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>The_Last_Bear.jpg</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -711,16 +711,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1155,7 +1155,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="57">
-      <c r="A2" s="18">
+      <c r="A2" s="16">
         <v>45887</v>
       </c>
       <c r="B2" s="13">
@@ -1165,13 +1165,13 @@
         <v>110</v>
       </c>
       <c r="D2" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="E2" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="10" t="s">
         <v>167</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>168</v>
       </c>
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
@@ -1183,7 +1183,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="57">
-      <c r="A3" s="18">
+      <c r="A3" s="16">
         <v>45999</v>
       </c>
       <c r="B3" s="13">
@@ -1193,13 +1193,13 @@
         <v>110</v>
       </c>
       <c r="D3" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>170</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>171</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -1221,13 +1221,13 @@
         <v>110</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>173</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>174</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -3860,13 +3860,13 @@
         <v>127</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E6" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="J6" t="s">
         <v>36</v>
@@ -3883,13 +3883,13 @@
         <v>127</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="J7" t="s">
         <v>36</v>
@@ -4016,10 +4016,10 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="C2 C3:C200" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="C8:C200 C2:C7" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"English,Math,Art,Science,Sports,Music,School,Community,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J2 J3:J200" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" sqref="J8:J200 J2:J7" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4324,13 +4324,13 @@
         <v>5</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="I6" s="4"/>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="14"/>
-      <c r="E7" s="17"/>
+      <c r="E7" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -4668,14 +4668,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="20.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="3" spans="1:6" ht="15">
       <c r="A3" s="1" t="s">

</xml_diff>

<commit_message>
Update Richard learning portfolio and images
</commit_message>
<xml_diff>
--- a/data/learning_portfolio.xlsx
+++ b/data/learning_portfolio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\88_YuHui\Streamlit\Richard_streamlit\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C02BA2-DFE4-4D77-994F-D29002145A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA0E498C-0C77-4E05-91EB-A1A5A8539F9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Profile" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="180">
   <si>
     <t>Field</t>
   </si>
@@ -154,9 +154,6 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>MATH KANGAROO TAIWAN</t>
-  </si>
-  <si>
     <t>Silver</t>
   </si>
   <si>
@@ -166,9 +163,6 @@
     <t>Richard participated in Math Kangaroo Taiwan and earned a Silver Award. This experience helped him build confidence in mathematical thinking and problem-solving.</t>
   </si>
   <si>
-    <t>award_001.jpg</t>
-  </si>
-  <si>
     <t>第63屆 奧林匹克數理競賽</t>
   </si>
   <si>
@@ -421,22 +415,13 @@
     <t>https://heyzine.com/flip-book/9991bced10.html</t>
   </si>
   <si>
-    <t>SMC Regional Round</t>
-  </si>
-  <si>
     <t>Marshall Cavendish Education (MCE)</t>
   </si>
   <si>
     <t>Richard earned a Silver Award in the SMC Regional Round. The competition encouraged him to think carefully, stay focused, and challenge himself in mathematics.</t>
   </si>
   <si>
-    <t>award_002.jpg</t>
-  </si>
-  <si>
     <t>Sports</t>
-  </si>
-  <si>
-    <t>Horizon Field Day – Boys' MVP</t>
   </si>
   <si>
     <t>Boys' MVP</t>
@@ -596,6 +581,26 @@
   </si>
   <si>
     <t>20261025_Performance.jpg</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>MATH KANGAROO TAIWAN</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>SMC Regional Round</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026_SMC_Regional_Round.jpg</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Horizon Field Day – Boys' MVP</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026_Horizon_Field_Day.jpg</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -879,6 +884,7 @@
         <name val="Carlito"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -897,7 +903,6 @@
         <name val="Carlito"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -978,17 +983,17 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="ReadingLogTable" displayName="ReadingLogTable" ref="A1:I6" dataDxfId="0" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="ReadingLogTable" displayName="ReadingLogTable" ref="A1:I6" dataDxfId="9" dataCellStyle="Normal">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Date" dataDxfId="9" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Year" dataDxfId="8" dataCellStyle="Normal"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="BookTitle" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Author" dataDxfId="6" dataCellStyle="Normal"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Category" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="Reflection" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Rating" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Image" dataDxfId="2" dataCellStyle="Normal"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="Link" dataDxfId="1" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Date" dataDxfId="8" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Year" dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="BookTitle" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Author" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Category" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="Reflection" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Rating" dataDxfId="2" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Image" dataDxfId="1" dataCellStyle="Normal"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="Link" dataDxfId="0" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1316,7 +1321,7 @@
         <v>23</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="H1" s="9" t="s">
         <v>25</v>
@@ -1336,16 +1341,16 @@
         <v>2025</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
@@ -1353,7 +1358,7 @@
         <v>36</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="57">
@@ -1364,16 +1369,16 @@
         <v>2025</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10"/>
@@ -1381,7 +1386,7 @@
         <v>36</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="57">
@@ -1392,16 +1397,16 @@
         <v>2025</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="G4" s="10"/>
       <c r="H4" s="10"/>
@@ -1409,7 +1414,7 @@
         <v>36</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="57">
@@ -1420,16 +1425,16 @@
         <v>2026</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="F5" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>112</v>
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="10"/>
@@ -1437,7 +1442,7 @@
         <v>36</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="42.75">
@@ -1448,16 +1453,16 @@
         <v>2026</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D6" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F6" s="10" t="s">
         <v>113</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>115</v>
       </c>
       <c r="G6" s="10"/>
       <c r="H6" s="10"/>
@@ -1465,7 +1470,7 @@
         <v>36</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -1476,16 +1481,16 @@
         <v>2026</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D7" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>116</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>118</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="10"/>
@@ -1493,7 +1498,7 @@
         <v>36</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="42.75">
@@ -1504,13 +1509,13 @@
         <v>2026</v>
       </c>
       <c r="C8" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>119</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>121</v>
       </c>
       <c r="F8" s="10"/>
       <c r="G8" s="10"/>
@@ -1519,7 +1524,7 @@
         <v>36</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="57">
@@ -1530,26 +1535,26 @@
         <v>2026</v>
       </c>
       <c r="C9" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="E9" s="13" t="s">
         <v>122</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>124</v>
       </c>
       <c r="F9" s="13"/>
       <c r="G9" s="13" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I9" s="13" t="s">
         <v>36</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -3952,20 +3957,18 @@
         <v>31</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>41</v>
-      </c>
+      <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4" t="s">
         <v>36</v>
@@ -3982,16 +3985,16 @@
         <v>31</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
@@ -4010,19 +4013,19 @@
         <v>31</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>126</v>
+        <v>176</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>129</v>
+        <v>177</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4" t="s">
@@ -4037,16 +4040,19 @@
         <v>2026</v>
       </c>
       <c r="C6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>131</v>
+        <v>178</v>
       </c>
       <c r="E6" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>133</v>
+        <v>128</v>
+      </c>
+      <c r="H6" t="s">
+        <v>179</v>
       </c>
       <c r="J6" t="s">
         <v>36</v>
@@ -4060,16 +4066,19 @@
         <v>2026</v>
       </c>
       <c r="C7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="E7" t="s">
         <v>130</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="E7" t="s">
-        <v>135</v>
-      </c>
       <c r="G7" s="13" t="s">
-        <v>136</v>
+        <v>131</v>
+      </c>
+      <c r="H7" t="s">
+        <v>179</v>
       </c>
       <c r="J7" t="s">
         <v>36</v>
@@ -4083,16 +4092,19 @@
         <v>2026</v>
       </c>
       <c r="C8" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="E8" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>139</v>
+        <v>134</v>
+      </c>
+      <c r="H8" t="s">
+        <v>179</v>
       </c>
       <c r="J8" t="s">
         <v>36</v>
@@ -4106,16 +4118,19 @@
         <v>2026</v>
       </c>
       <c r="C9" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="E9" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>141</v>
+        <v>136</v>
+      </c>
+      <c r="H9" t="s">
+        <v>179</v>
       </c>
       <c r="J9" t="s">
         <v>36</v>
@@ -4129,16 +4144,19 @@
         <v>2026</v>
       </c>
       <c r="C10" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="E10" t="s">
+        <v>133</v>
+      </c>
+      <c r="G10" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="G10" s="13" t="s">
-        <v>143</v>
+      <c r="H10" t="s">
+        <v>179</v>
       </c>
       <c r="J10" t="s">
         <v>36</v>
@@ -4152,16 +4170,19 @@
         <v>2026</v>
       </c>
       <c r="C11" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E11" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>145</v>
+        <v>140</v>
+      </c>
+      <c r="H11" t="s">
+        <v>179</v>
       </c>
       <c r="J11" t="s">
         <v>36</v>
@@ -4175,19 +4196,19 @@
         <v>2026</v>
       </c>
       <c r="C12" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E12" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="F12" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J12" t="s">
         <v>36</v>
@@ -4236,19 +4257,19 @@
         <v>21</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>24</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>25</v>
@@ -4265,17 +4286,17 @@
         <v>2026</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -4291,16 +4312,16 @@
         <v>2026</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -4350,10 +4371,10 @@
         <v>20</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>21</v>
@@ -4362,7 +4383,7 @@
         <v>23</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>24</v>
@@ -4379,20 +4400,20 @@
         <v>2025</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4">
         <v>5</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -4404,20 +4425,20 @@
         <v>2025</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="4">
         <v>5</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -4429,20 +4450,20 @@
         <v>2026</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4">
         <v>5</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="I4" s="4"/>
     </row>
@@ -4454,20 +4475,20 @@
         <v>2026</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4">
         <v>5</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="I5" s="4"/>
     </row>
@@ -4479,20 +4500,20 @@
         <v>2026</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4">
         <v>5</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="I6" s="4"/>
     </row>
@@ -4528,25 +4549,25 @@
         <v>20</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -4572,7 +4593,7 @@
         <v>4</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -4598,7 +4619,7 @@
         <v>4</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -4624,7 +4645,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -4655,22 +4676,22 @@
         <v>20</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.5">
@@ -4678,22 +4699,22 @@
         <v>2026</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>76</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -4701,19 +4722,19 @@
         <v>2025</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="G3" s="4"/>
     </row>
@@ -4741,43 +4762,43 @@
         <v>21</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="28.5">
       <c r="A2" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="28.5">
       <c r="A3" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -4785,10 +4806,10 @@
         <v>26</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -4796,21 +4817,21 @@
         <v>27</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -4833,7 +4854,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20.25">
       <c r="A1" s="14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -4843,15 +4864,15 @@
     </row>
     <row r="3" spans="1:6" ht="15">
       <c r="A3" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B4" s="3">
         <f>COUNTA(LearningTimeline!D2:D200)</f>
@@ -4860,7 +4881,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B5" s="3">
         <f>COUNTIF(LearningTimeline!I2:I200,"Yes")</f>
@@ -4869,7 +4890,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B6" s="3">
         <f>COUNTA(Awards!D2:D200)</f>
@@ -4878,7 +4899,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B7" s="3">
         <f>COUNTA(Projects!D2:D199)</f>
@@ -4887,7 +4908,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B8" s="3">
         <f>COUNTA(ReadingLog!C2:C201)</f>
@@ -4896,7 +4917,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B9" s="3">
         <f>IFERROR(AVERAGE(ReadingLog!G2:G201),0)</f>

</xml_diff>